<commit_message>
WIP: Added namespaces for Sector
</commit_message>
<xml_diff>
--- a/code/vocab_csv/namespaces.xlsx
+++ b/code/vocab_csv/namespaces.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="337">
   <si>
     <t>preffix</t>
   </si>
@@ -526,6 +526,60 @@
   </si>
   <si>
     <t>Laws and Authorities for US</t>
+  </si>
+  <si>
+    <t>sector-education</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/education#</t>
+  </si>
+  <si>
+    <t>Education Sector</t>
+  </si>
+  <si>
+    <t>sector-finance</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/finance#</t>
+  </si>
+  <si>
+    <t>Finance Sector</t>
+  </si>
+  <si>
+    <t>sector-health</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/health#</t>
+  </si>
+  <si>
+    <t>Health Sector</t>
+  </si>
+  <si>
+    <t>sector-infra</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/infra#</t>
+  </si>
+  <si>
+    <t>Infrastructure Sector</t>
+  </si>
+  <si>
+    <t>sector-law</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/law#</t>
+  </si>
+  <si>
+    <t>Law Enforcement and Justice Sector</t>
+  </si>
+  <si>
+    <t>sector-publicservices</t>
+  </si>
+  <si>
+    <t>https://w3id.org/dpv/sector/publicservices#</t>
+  </si>
+  <si>
+    <t>Public Services Sector</t>
   </si>
   <si>
     <t>dct</t>
@@ -1169,7 +1223,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1238,6 +1292,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -2499,6 +2556,108 @@
         <v>11</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D57" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D58" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D59" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D61" s="23">
+        <v>45627.0</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B2"/>
@@ -2557,8 +2716,14 @@
     <hyperlink r:id="rId54" ref="B53"/>
     <hyperlink r:id="rId55" ref="B54"/>
     <hyperlink r:id="rId56" ref="B55"/>
+    <hyperlink r:id="rId57" ref="B56"/>
+    <hyperlink r:id="rId58" ref="B57"/>
+    <hyperlink r:id="rId59" ref="B58"/>
+    <hyperlink r:id="rId60" ref="B59"/>
+    <hyperlink r:id="rId61" ref="B60"/>
+    <hyperlink r:id="rId62" ref="B61"/>
   </hyperlinks>
-  <drawing r:id="rId57"/>
+  <drawing r:id="rId63"/>
 </worksheet>
 </file>
 
@@ -2600,537 +2765,537 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>173</v>
-      </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
-      <c r="V2" s="25"/>
+      <c r="A2" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
     </row>
     <row r="3">
-      <c r="A3" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>175</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="25"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="25"/>
-      <c r="S3" s="25"/>
-      <c r="T3" s="25"/>
-      <c r="U3" s="25"/>
-      <c r="V3" s="25"/>
+      <c r="A3" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="25"/>
-      <c r="N4" s="25"/>
-      <c r="O4" s="25"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="25"/>
-      <c r="R4" s="25"/>
-      <c r="S4" s="25"/>
-      <c r="T4" s="25"/>
-      <c r="U4" s="25"/>
-      <c r="V4" s="25"/>
+      <c r="A4" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="26"/>
+      <c r="T4" s="26"/>
+      <c r="U4" s="26"/>
+      <c r="V4" s="26"/>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
-      <c r="O5" s="25"/>
-      <c r="P5" s="25"/>
-      <c r="Q5" s="25"/>
-      <c r="R5" s="25"/>
-      <c r="S5" s="25"/>
-      <c r="T5" s="25"/>
-      <c r="U5" s="25"/>
-      <c r="V5" s="25"/>
+      <c r="A5" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
+      <c r="Q5" s="26"/>
+      <c r="R5" s="26"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="26"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="25"/>
-      <c r="U6" s="25"/>
-      <c r="V6" s="25"/>
+      <c r="A6" s="27" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="26"/>
+      <c r="T6" s="26"/>
+      <c r="U6" s="26"/>
+      <c r="V6" s="26"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>187</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="25"/>
-      <c r="S7" s="25"/>
-      <c r="T7" s="25"/>
-      <c r="U7" s="25"/>
-      <c r="V7" s="25"/>
+      <c r="A7" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="C8" s="29" t="str">
+      <c r="A8" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="C8" s="30" t="str">
         <f>HYPERLINK("https://www.specialprivacy.eu/images/documents/SPECIAL_D25_M21_V10.pdf","SPECIAL Log vocabulary cf. SPECIAL Deliverable D2.5")</f>
         <v>SPECIAL Log vocabulary cf. SPECIAL Deliverable D2.5</v>
       </c>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-      <c r="M8" s="25"/>
-      <c r="N8" s="25"/>
-      <c r="O8" s="25"/>
-      <c r="P8" s="25"/>
-      <c r="Q8" s="25"/>
-      <c r="R8" s="25"/>
-      <c r="S8" s="25"/>
-      <c r="T8" s="25"/>
-      <c r="U8" s="25"/>
-      <c r="V8" s="25"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
+      <c r="N8" s="26"/>
+      <c r="O8" s="26"/>
+      <c r="P8" s="26"/>
+      <c r="Q8" s="26"/>
+      <c r="R8" s="26"/>
+      <c r="S8" s="26"/>
+      <c r="T8" s="26"/>
+      <c r="U8" s="26"/>
+      <c r="V8" s="26"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>192</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
-      <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="25"/>
-      <c r="R9" s="25"/>
-      <c r="S9" s="25"/>
-      <c r="T9" s="25"/>
-      <c r="U9" s="25"/>
-      <c r="V9" s="25"/>
+      <c r="A9" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="26"/>
+      <c r="S9" s="26"/>
+      <c r="T9" s="26"/>
+      <c r="U9" s="26"/>
+      <c r="V9" s="26"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="s">
-        <v>194</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="25"/>
-      <c r="M10" s="25"/>
-      <c r="N10" s="25"/>
-      <c r="O10" s="25"/>
-      <c r="P10" s="25"/>
-      <c r="Q10" s="25"/>
-      <c r="R10" s="25"/>
-      <c r="S10" s="25"/>
-      <c r="T10" s="25"/>
-      <c r="U10" s="25"/>
-      <c r="V10" s="25"/>
+      <c r="A10" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="26"/>
+      <c r="M10" s="26"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="26"/>
+      <c r="P10" s="26"/>
+      <c r="Q10" s="26"/>
+      <c r="R10" s="26"/>
+      <c r="S10" s="26"/>
+      <c r="T10" s="26"/>
+      <c r="U10" s="26"/>
+      <c r="V10" s="26"/>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="25"/>
-      <c r="U11" s="25"/>
-      <c r="V11" s="25"/>
+      <c r="A11" s="32" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="26"/>
+      <c r="P11" s="26"/>
+      <c r="Q11" s="26"/>
+      <c r="R11" s="26"/>
+      <c r="S11" s="26"/>
+      <c r="T11" s="26"/>
+      <c r="U11" s="26"/>
+      <c r="V11" s="26"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>200</v>
-      </c>
-      <c r="B12" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>202</v>
-      </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="25"/>
-      <c r="R12" s="25"/>
-      <c r="S12" s="25"/>
-      <c r="T12" s="25"/>
-      <c r="U12" s="25"/>
-      <c r="V12" s="25"/>
+      <c r="A12" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>219</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="26"/>
+      <c r="P12" s="26"/>
+      <c r="Q12" s="26"/>
+      <c r="R12" s="26"/>
+      <c r="S12" s="26"/>
+      <c r="T12" s="26"/>
+      <c r="U12" s="26"/>
+      <c r="V12" s="26"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="30" t="s">
-        <v>204</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="25"/>
-      <c r="R13" s="25"/>
-      <c r="S13" s="25"/>
-      <c r="T13" s="25"/>
-      <c r="U13" s="25"/>
-      <c r="V13" s="25"/>
+      <c r="A13" s="24" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>222</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>223</v>
+      </c>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="26"/>
+      <c r="M13" s="26"/>
+      <c r="N13" s="26"/>
+      <c r="O13" s="26"/>
+      <c r="P13" s="26"/>
+      <c r="Q13" s="26"/>
+      <c r="R13" s="26"/>
+      <c r="S13" s="26"/>
+      <c r="T13" s="26"/>
+      <c r="U13" s="26"/>
+      <c r="V13" s="26"/>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>207</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>208</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="25"/>
-      <c r="N14" s="25"/>
-      <c r="O14" s="25"/>
-      <c r="P14" s="25"/>
-      <c r="Q14" s="25"/>
-      <c r="R14" s="25"/>
-      <c r="S14" s="25"/>
-      <c r="T14" s="25"/>
-      <c r="U14" s="25"/>
-      <c r="V14" s="25"/>
+      <c r="A14" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>225</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="26"/>
+      <c r="Q14" s="26"/>
+      <c r="R14" s="26"/>
+      <c r="S14" s="26"/>
+      <c r="T14" s="26"/>
+      <c r="U14" s="26"/>
+      <c r="V14" s="26"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>210</v>
+        <v>228</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="B24" s="32" t="s">
-        <v>235</v>
+        <v>252</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>253</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -3174,13 +3339,13 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="s">
-        <v>246</v>
+      <c r="A1" s="34" t="s">
+        <v>264</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="C1" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="C1" s="35" t="s">
         <v>28</v>
       </c>
       <c r="D1" s="8">
@@ -3194,14 +3359,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="s">
-        <v>248</v>
+      <c r="A2" s="36" t="s">
+        <v>266</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>250</v>
+        <v>267</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>268</v>
       </c>
       <c r="D2" s="8">
         <v>44601.0</v>
@@ -3215,13 +3380,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="D3" s="8">
         <v>44601.0</v>
@@ -3235,13 +3400,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="D4" s="8">
         <v>44727.0</v>
@@ -3250,18 +3415,18 @@
         <v>11</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="D5" s="8">
         <v>44650.0</v>
@@ -3270,34 +3435,34 @@
         <v>11</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="6" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="H6" s="6"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="D7" s="8">
         <v>44601.0</v>
@@ -3310,14 +3475,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="35" t="s">
-        <v>269</v>
+      <c r="A8" s="36" t="s">
+        <v>287</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>271</v>
+        <v>288</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>289</v>
       </c>
       <c r="D8" s="8">
         <v>44601.0</v>
@@ -3331,13 +3496,13 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
       <c r="D9" s="8">
         <v>44601.0</v>
@@ -3351,13 +3516,13 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="D10" s="8">
         <v>44727.0</v>
@@ -3366,18 +3531,18 @@
         <v>11</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="D11" s="8">
         <v>44650.0</v>
@@ -3386,18 +3551,18 @@
         <v>11</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="D12" s="8">
         <v>44650.0</v>
@@ -3406,18 +3571,18 @@
         <v>11</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="D13" s="8">
         <v>44601.0</v>
@@ -3430,14 +3595,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="35" t="s">
-        <v>287</v>
+      <c r="A14" s="36" t="s">
+        <v>305</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>289</v>
+        <v>306</v>
+      </c>
+      <c r="C14" s="35" t="s">
+        <v>307</v>
       </c>
       <c r="D14" s="8">
         <v>44601.0</v>
@@ -3451,13 +3616,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
       <c r="D15" s="8">
         <v>44601.0</v>
@@ -3471,13 +3636,13 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="D16" s="8">
         <v>44727.0</v>
@@ -3486,18 +3651,18 @@
         <v>11</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="D17" s="8">
         <v>44650.0</v>
@@ -3506,18 +3671,18 @@
         <v>11</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
       <c r="D18" s="8">
         <v>44650.0</v>
@@ -3526,18 +3691,18 @@
         <v>11</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>302</v>
+        <v>320</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="D19" s="8">
         <v>44734.0</v>
@@ -3551,13 +3716,13 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="D20" s="8">
         <v>44734.0</v>
@@ -3570,146 +3735,146 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="36" t="s">
-        <v>308</v>
-      </c>
-      <c r="B21" s="37" t="s">
+      <c r="A21" s="37" t="s">
+        <v>326</v>
+      </c>
+      <c r="B21" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="36" t="s">
-        <v>309</v>
-      </c>
-      <c r="D21" s="38">
+      <c r="C21" s="37" t="s">
+        <v>327</v>
+      </c>
+      <c r="D21" s="39">
         <v>44734.0</v>
       </c>
-      <c r="E21" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="39" t="s">
+      <c r="E21" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="36"/>
-      <c r="R21" s="36"/>
-      <c r="S21" s="36"/>
-      <c r="T21" s="36"/>
-      <c r="U21" s="36"/>
-      <c r="V21" s="36"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="37"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="37"/>
+      <c r="Q21" s="37"/>
+      <c r="R21" s="37"/>
+      <c r="S21" s="37"/>
+      <c r="T21" s="37"/>
+      <c r="U21" s="37"/>
+      <c r="V21" s="37"/>
     </row>
     <row r="22">
-      <c r="A22" s="36" t="s">
-        <v>310</v>
-      </c>
-      <c r="B22" s="37" t="s">
-        <v>311</v>
-      </c>
-      <c r="C22" s="36" t="s">
-        <v>312</v>
-      </c>
-      <c r="D22" s="38">
+      <c r="A22" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="B22" s="38" t="s">
+        <v>329</v>
+      </c>
+      <c r="C22" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="D22" s="39">
         <v>44734.0</v>
       </c>
-      <c r="E22" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="39" t="s">
+      <c r="E22" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="36"/>
-      <c r="N22" s="36"/>
-      <c r="O22" s="36"/>
-      <c r="P22" s="36"/>
-      <c r="Q22" s="36"/>
-      <c r="R22" s="36"/>
-      <c r="S22" s="36"/>
-      <c r="T22" s="36"/>
-      <c r="U22" s="36"/>
-      <c r="V22" s="36"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="37"/>
+      <c r="K22" s="37"/>
+      <c r="L22" s="37"/>
+      <c r="M22" s="37"/>
+      <c r="N22" s="37"/>
+      <c r="O22" s="37"/>
+      <c r="P22" s="37"/>
+      <c r="Q22" s="37"/>
+      <c r="R22" s="37"/>
+      <c r="S22" s="37"/>
+      <c r="T22" s="37"/>
+      <c r="U22" s="37"/>
+      <c r="V22" s="37"/>
     </row>
     <row r="23">
-      <c r="A23" s="36" t="s">
-        <v>313</v>
-      </c>
-      <c r="B23" s="37" t="s">
-        <v>314</v>
-      </c>
-      <c r="C23" s="36" t="s">
-        <v>315</v>
-      </c>
-      <c r="D23" s="38">
+      <c r="A23" s="37" t="s">
+        <v>331</v>
+      </c>
+      <c r="B23" s="38" t="s">
+        <v>332</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>333</v>
+      </c>
+      <c r="D23" s="39">
         <v>44734.0</v>
       </c>
-      <c r="E23" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="39" t="s">
+      <c r="E23" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
-      <c r="O23" s="36"/>
-      <c r="P23" s="36"/>
-      <c r="Q23" s="36"/>
-      <c r="R23" s="36"/>
-      <c r="S23" s="36"/>
-      <c r="T23" s="36"/>
-      <c r="U23" s="36"/>
-      <c r="V23" s="36"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="37"/>
+      <c r="P23" s="37"/>
+      <c r="Q23" s="37"/>
+      <c r="R23" s="37"/>
+      <c r="S23" s="37"/>
+      <c r="T23" s="37"/>
+      <c r="U23" s="37"/>
+      <c r="V23" s="37"/>
     </row>
     <row r="24">
-      <c r="A24" s="36" t="s">
-        <v>316</v>
-      </c>
-      <c r="B24" s="37" t="s">
-        <v>317</v>
-      </c>
-      <c r="C24" s="36" t="s">
-        <v>318</v>
-      </c>
-      <c r="D24" s="38">
+      <c r="A24" s="37" t="s">
+        <v>334</v>
+      </c>
+      <c r="B24" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="C24" s="37" t="s">
+        <v>336</v>
+      </c>
+      <c r="D24" s="39">
         <v>45189.0</v>
       </c>
-      <c r="E24" s="36" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="36"/>
-      <c r="R24" s="36"/>
-      <c r="S24" s="36"/>
-      <c r="T24" s="36"/>
-      <c r="U24" s="36"/>
-      <c r="V24" s="36"/>
+      <c r="E24" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
+      <c r="O24" s="37"/>
+      <c r="P24" s="37"/>
+      <c r="Q24" s="37"/>
+      <c r="R24" s="37"/>
+      <c r="S24" s="37"/>
+      <c r="T24" s="37"/>
+      <c r="U24" s="37"/>
+      <c r="V24" s="37"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>